<commit_message>
Docs, build prompt pack and feature-gap sheet updated to 0.9.1
- User's Guide, Quick Start, Technical System Design and Developer's Guide (Markdown and Word): macOS and Linux
  install, the platform design, the loose-date import fix
- Build prompt pack: version 0.9.1, release file names, arm64 Linux, the Linux universal-merge method, §6.16
- Feature-gap sheet: cross-platform done in 0.9.0, the import fix in 0.9.1

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KZ8RpfjgQtZthigNSkA5xL
</commit_message>
<xml_diff>
--- a/docs/feature-gaps.xlsx
+++ b/docs/feature-gaps.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current app extras" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Feature gaps'!$A$4:$L$64</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Feature gaps'!$A$4:$L$65</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -656,15 +656,15 @@
         <v>1</v>
       </c>
       <c r="D5" s="4">
-        <f>COUNTIFS('Feature gaps'!$F$5:$F$64,A5,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done")</f>
+        <f>COUNTIFS('Feature gaps'!$F$5:$F$65,A5,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="E5" s="6">
-        <f>SUMIFS('Feature gaps'!$G$5:$G$64,'Feature gaps'!$F$5:$F$64,A5,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done")</f>
+        <f>SUMIFS('Feature gaps'!$G$5:$G$65,'Feature gaps'!$F$5:$F$65,A5,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="F5" s="6">
-        <f>SUMIFS('Feature gaps'!$H$5:$H$64,'Feature gaps'!$F$5:$F$64,A5,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done")</f>
+        <f>SUMIFS('Feature gaps'!$H$5:$H$65,'Feature gaps'!$F$5:$F$65,A5,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -686,15 +686,15 @@
         <v>3</v>
       </c>
       <c r="D6" s="4">
-        <f>COUNTIFS('Feature gaps'!$F$5:$F$64,A6,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done")</f>
+        <f>COUNTIFS('Feature gaps'!$F$5:$F$65,A6,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="E6" s="6">
-        <f>SUMIFS('Feature gaps'!$G$5:$G$64,'Feature gaps'!$F$5:$F$64,A6,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done")</f>
+        <f>SUMIFS('Feature gaps'!$G$5:$G$65,'Feature gaps'!$F$5:$F$65,A6,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="F6" s="6">
-        <f>SUMIFS('Feature gaps'!$H$5:$H$64,'Feature gaps'!$F$5:$F$64,A6,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done")</f>
+        <f>SUMIFS('Feature gaps'!$H$5:$H$65,'Feature gaps'!$F$5:$F$65,A6,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -716,15 +716,15 @@
         <v>5</v>
       </c>
       <c r="D7" s="4">
-        <f>COUNTIFS('Feature gaps'!$F$5:$F$64,A7,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done")</f>
+        <f>COUNTIFS('Feature gaps'!$F$5:$F$65,A7,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="E7" s="6">
-        <f>SUMIFS('Feature gaps'!$G$5:$G$64,'Feature gaps'!$F$5:$F$64,A7,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done")</f>
+        <f>SUMIFS('Feature gaps'!$G$5:$G$65,'Feature gaps'!$F$5:$F$65,A7,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="F7" s="6">
-        <f>SUMIFS('Feature gaps'!$H$5:$H$64,'Feature gaps'!$F$5:$F$64,A7,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done")</f>
+        <f>SUMIFS('Feature gaps'!$H$5:$H$65,'Feature gaps'!$F$5:$F$65,A7,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -746,15 +746,15 @@
         <v>10</v>
       </c>
       <c r="D8" s="4">
-        <f>COUNTIFS('Feature gaps'!$F$5:$F$64,A8,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done")</f>
+        <f>COUNTIFS('Feature gaps'!$F$5:$F$65,A8,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="E8" s="6">
-        <f>SUMIFS('Feature gaps'!$G$5:$G$64,'Feature gaps'!$F$5:$F$64,A8,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done")</f>
+        <f>SUMIFS('Feature gaps'!$G$5:$G$65,'Feature gaps'!$F$5:$F$65,A8,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="F8" s="6">
-        <f>SUMIFS('Feature gaps'!$H$5:$H$64,'Feature gaps'!$F$5:$F$64,A8,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done")</f>
+        <f>SUMIFS('Feature gaps'!$H$5:$H$65,'Feature gaps'!$F$5:$F$65,A8,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -776,15 +776,15 @@
         <v>15</v>
       </c>
       <c r="D9" s="4">
-        <f>COUNTIFS('Feature gaps'!$F$5:$F$64,A9,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done")</f>
+        <f>COUNTIFS('Feature gaps'!$F$5:$F$65,A9,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="E9" s="6">
-        <f>SUMIFS('Feature gaps'!$G$5:$G$64,'Feature gaps'!$F$5:$F$64,A9,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done")</f>
+        <f>SUMIFS('Feature gaps'!$G$5:$G$65,'Feature gaps'!$F$5:$F$65,A9,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="F9" s="6">
-        <f>SUMIFS('Feature gaps'!$H$5:$H$64,'Feature gaps'!$F$5:$F$64,A9,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done")</f>
+        <f>SUMIFS('Feature gaps'!$H$5:$H$65,'Feature gaps'!$F$5:$F$65,A9,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -806,15 +806,15 @@
         <v>30</v>
       </c>
       <c r="D10" s="4">
-        <f>COUNTIFS('Feature gaps'!$F$5:$F$64,A10,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done")</f>
+        <f>COUNTIFS('Feature gaps'!$F$5:$F$65,A10,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="E10" s="6">
-        <f>SUMIFS('Feature gaps'!$G$5:$G$64,'Feature gaps'!$F$5:$F$64,A10,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done")</f>
+        <f>SUMIFS('Feature gaps'!$G$5:$G$65,'Feature gaps'!$F$5:$F$65,A10,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="F10" s="6">
-        <f>SUMIFS('Feature gaps'!$H$5:$H$64,'Feature gaps'!$F$5:$F$64,A10,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done")</f>
+        <f>SUMIFS('Feature gaps'!$H$5:$H$65,'Feature gaps'!$F$5:$F$65,A10,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -836,15 +836,15 @@
         <v>0</v>
       </c>
       <c r="D11" s="4">
-        <f>COUNTIFS('Feature gaps'!$F$5:$F$64,A11,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done")</f>
+        <f>COUNTIFS('Feature gaps'!$F$5:$F$65,A11,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="E11" s="6">
-        <f>SUMIFS('Feature gaps'!$G$5:$G$64,'Feature gaps'!$F$5:$F$64,A11,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done")</f>
+        <f>SUMIFS('Feature gaps'!$G$5:$G$65,'Feature gaps'!$F$5:$F$65,A11,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="F11" s="6">
-        <f>SUMIFS('Feature gaps'!$H$5:$H$64,'Feature gaps'!$F$5:$F$64,A11,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done")</f>
+        <f>SUMIFS('Feature gaps'!$H$5:$H$65,'Feature gaps'!$F$5:$F$65,A11,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -917,15 +917,15 @@
       </c>
       <c r="C15" s="9" t="n"/>
       <c r="D15" s="9">
-        <f>COUNTIFS('Feature gaps'!$J$5:$J$64,A15,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done")</f>
+        <f>COUNTIFS('Feature gaps'!$J$5:$J$65,A15,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>SUMIFS('Feature gaps'!$G$5:$G$64,'Feature gaps'!$J$5:$J$64,A15,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done")</f>
+        <f>SUMIFS('Feature gaps'!$G$5:$G$65,'Feature gaps'!$J$5:$J$65,A15,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>SUMIFS('Feature gaps'!$H$5:$H$64,'Feature gaps'!$J$5:$J$64,A15,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done")</f>
+        <f>SUMIFS('Feature gaps'!$H$5:$H$65,'Feature gaps'!$J$5:$J$65,A15,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done")</f>
         <v/>
       </c>
     </row>
@@ -942,15 +942,15 @@
       </c>
       <c r="C16" s="9" t="n"/>
       <c r="D16" s="9">
-        <f>COUNTIFS('Feature gaps'!$J$5:$J$64,A16,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done")</f>
+        <f>COUNTIFS('Feature gaps'!$J$5:$J$65,A16,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="E16" s="10">
-        <f>SUMIFS('Feature gaps'!$G$5:$G$64,'Feature gaps'!$J$5:$J$64,A16,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done")</f>
+        <f>SUMIFS('Feature gaps'!$G$5:$G$65,'Feature gaps'!$J$5:$J$65,A16,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="F16" s="10">
-        <f>SUMIFS('Feature gaps'!$H$5:$H$64,'Feature gaps'!$J$5:$J$64,A16,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done")</f>
+        <f>SUMIFS('Feature gaps'!$H$5:$H$65,'Feature gaps'!$J$5:$J$65,A16,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done")</f>
         <v/>
       </c>
     </row>
@@ -967,15 +967,15 @@
       </c>
       <c r="C17" s="9" t="n"/>
       <c r="D17" s="9">
-        <f>COUNTIFS('Feature gaps'!$J$5:$J$64,A17,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done")</f>
+        <f>COUNTIFS('Feature gaps'!$J$5:$J$65,A17,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>SUMIFS('Feature gaps'!$G$5:$G$64,'Feature gaps'!$J$5:$J$64,A17,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done")</f>
+        <f>SUMIFS('Feature gaps'!$G$5:$G$65,'Feature gaps'!$J$5:$J$65,A17,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>SUMIFS('Feature gaps'!$H$5:$H$64,'Feature gaps'!$J$5:$J$64,A17,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done")</f>
+        <f>SUMIFS('Feature gaps'!$H$5:$H$65,'Feature gaps'!$J$5:$J$65,A17,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done")</f>
         <v/>
       </c>
     </row>
@@ -992,15 +992,15 @@
       </c>
       <c r="C18" s="9" t="n"/>
       <c r="D18" s="9">
-        <f>COUNTIFS('Feature gaps'!$J$5:$J$64,A18,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done")</f>
+        <f>COUNTIFS('Feature gaps'!$J$5:$J$65,A18,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="E18" s="10">
-        <f>SUMIFS('Feature gaps'!$G$5:$G$64,'Feature gaps'!$J$5:$J$64,A18,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done")</f>
+        <f>SUMIFS('Feature gaps'!$G$5:$G$65,'Feature gaps'!$J$5:$J$65,A18,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="F18" s="10">
-        <f>SUMIFS('Feature gaps'!$H$5:$H$64,'Feature gaps'!$J$5:$J$64,A18,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done")</f>
+        <f>SUMIFS('Feature gaps'!$H$5:$H$65,'Feature gaps'!$J$5:$J$65,A18,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done")</f>
         <v/>
       </c>
     </row>
@@ -1017,15 +1017,15 @@
       </c>
       <c r="C19" s="9" t="n"/>
       <c r="D19" s="9">
-        <f>COUNTIFS('Feature gaps'!$J$5:$J$64,A19,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done")</f>
+        <f>COUNTIFS('Feature gaps'!$J$5:$J$65,A19,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>SUMIFS('Feature gaps'!$G$5:$G$64,'Feature gaps'!$J$5:$J$64,A19,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done")</f>
+        <f>SUMIFS('Feature gaps'!$G$5:$G$65,'Feature gaps'!$J$5:$J$65,A19,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>SUMIFS('Feature gaps'!$H$5:$H$64,'Feature gaps'!$J$5:$J$64,A19,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done")</f>
+        <f>SUMIFS('Feature gaps'!$H$5:$H$65,'Feature gaps'!$J$5:$J$65,A19,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done")</f>
         <v/>
       </c>
     </row>
@@ -1042,15 +1042,15 @@
       </c>
       <c r="C20" s="9" t="n"/>
       <c r="D20" s="9">
-        <f>COUNTIFS('Feature gaps'!$J$5:$J$64,A20,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done")</f>
+        <f>COUNTIFS('Feature gaps'!$J$5:$J$65,A20,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="E20" s="10">
-        <f>SUMIFS('Feature gaps'!$G$5:$G$64,'Feature gaps'!$J$5:$J$64,A20,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done")</f>
+        <f>SUMIFS('Feature gaps'!$G$5:$G$65,'Feature gaps'!$J$5:$J$65,A20,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="F20" s="10">
-        <f>SUMIFS('Feature gaps'!$H$5:$H$64,'Feature gaps'!$J$5:$J$64,A20,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done")</f>
+        <f>SUMIFS('Feature gaps'!$H$5:$H$65,'Feature gaps'!$J$5:$J$65,A20,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done")</f>
         <v/>
       </c>
     </row>
@@ -1078,7 +1078,7 @@
         </is>
       </c>
       <c r="D23" s="11">
-        <f>COUNTIF('Feature gaps'!$K$5:$K$64,A23)</f>
+        <f>COUNTIF('Feature gaps'!$K$5:$K$65,A23)</f>
         <v/>
       </c>
     </row>
@@ -1089,7 +1089,7 @@
         </is>
       </c>
       <c r="D24" s="11">
-        <f>COUNTIF('Feature gaps'!$K$5:$K$64,A24)</f>
+        <f>COUNTIF('Feature gaps'!$K$5:$K$65,A24)</f>
         <v/>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="D25" s="11">
-        <f>COUNTIF('Feature gaps'!$K$5:$K$64,A25)</f>
+        <f>COUNTIF('Feature gaps'!$K$5:$K$65,A25)</f>
         <v/>
       </c>
     </row>
@@ -1111,7 +1111,7 @@
         </is>
       </c>
       <c r="D26" s="11">
-        <f>COUNTIF('Feature gaps'!$K$5:$K$64,A26)</f>
+        <f>COUNTIF('Feature gaps'!$K$5:$K$65,A26)</f>
         <v/>
       </c>
     </row>
@@ -1122,7 +1122,7 @@
         </is>
       </c>
       <c r="D27" s="11">
-        <f>COUNTIF('Feature gaps'!$K$5:$K$64,A27)</f>
+        <f>COUNTIF('Feature gaps'!$K$5:$K$65,A27)</f>
         <v/>
       </c>
     </row>
@@ -1164,11 +1164,11 @@
       <c r="B30" s="11" t="n"/>
       <c r="C30" s="11" t="n"/>
       <c r="D30" s="11">
-        <f>COUNTIF('Feature gaps'!$C$5:$C$64,A30)</f>
+        <f>COUNTIF('Feature gaps'!$C$5:$C$65,A30)</f>
         <v/>
       </c>
       <c r="E30" s="11">
-        <f>COUNTIFS('Feature gaps'!$C$5:$C$64,A30,'Feature gaps'!$K$5:$K$64,"Done")</f>
+        <f>COUNTIFS('Feature gaps'!$C$5:$C$65,A30,'Feature gaps'!$K$5:$K$65,"Done")</f>
         <v/>
       </c>
       <c r="F30" s="11">
@@ -1176,7 +1176,7 @@
         <v/>
       </c>
       <c r="G30" s="11">
-        <f>TEXT(SUMIFS('Feature gaps'!$G$5:$G$64,'Feature gaps'!$C$5:$C$64,A30,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done"),"0.0")&amp;" – "&amp;TEXT(SUMIFS('Feature gaps'!$H$5:$H$64,'Feature gaps'!$C$5:$C$64,A30,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done"),"0")</f>
+        <f>TEXT(SUMIFS('Feature gaps'!$G$5:$G$65,'Feature gaps'!$C$5:$C$65,A30,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done"),"0.0")&amp;" – "&amp;TEXT(SUMIFS('Feature gaps'!$H$5:$H$65,'Feature gaps'!$C$5:$C$65,A30,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done"),"0")</f>
         <v/>
       </c>
     </row>
@@ -1189,11 +1189,11 @@
       <c r="B31" s="11" t="n"/>
       <c r="C31" s="11" t="n"/>
       <c r="D31" s="11">
-        <f>COUNTIF('Feature gaps'!$C$5:$C$64,A31)</f>
+        <f>COUNTIF('Feature gaps'!$C$5:$C$65,A31)</f>
         <v/>
       </c>
       <c r="E31" s="11">
-        <f>COUNTIFS('Feature gaps'!$C$5:$C$64,A31,'Feature gaps'!$K$5:$K$64,"Done")</f>
+        <f>COUNTIFS('Feature gaps'!$C$5:$C$65,A31,'Feature gaps'!$K$5:$K$65,"Done")</f>
         <v/>
       </c>
       <c r="F31" s="11">
@@ -1201,7 +1201,7 @@
         <v/>
       </c>
       <c r="G31" s="11">
-        <f>TEXT(SUMIFS('Feature gaps'!$G$5:$G$64,'Feature gaps'!$C$5:$C$64,A31,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done"),"0.0")&amp;" – "&amp;TEXT(SUMIFS('Feature gaps'!$H$5:$H$64,'Feature gaps'!$C$5:$C$64,A31,'Feature gaps'!$K$5:$K$64,"&lt;&gt;Done"),"0")</f>
+        <f>TEXT(SUMIFS('Feature gaps'!$G$5:$G$65,'Feature gaps'!$C$5:$C$65,A31,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done"),"0.0")&amp;" – "&amp;TEXT(SUMIFS('Feature gaps'!$H$5:$H$65,'Feature gaps'!$C$5:$C$65,A31,'Feature gaps'!$K$5:$K$65,"&lt;&gt;Done"),"0")</f>
         <v/>
       </c>
     </row>
@@ -1255,7 +1255,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L64"/>
+  <dimension ref="A1:L65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1275,7 +1275,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>The original ReminderFox add-on (2.1.6) and ReminderFoxAgain 0.8.1 — ReminderFox's features still to bring across, and new features (proposed or added)</t>
+          <t>The original ReminderFox add-on (2.1.6) and ReminderFoxAgain 0.9.1 — ReminderFox's features still to bring across, and new features (proposed or added)</t>
         </is>
       </c>
     </row>
@@ -1309,7 +1309,7 @@
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>Current app (0.8.1)</t>
+          <t>Current app (0.9.1)</t>
         </is>
       </c>
       <c r="F4" s="14" t="inlineStr">
@@ -4073,7 +4073,7 @@
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>Windows only</t>
+          <t>Done in 0.9.0</t>
         </is>
       </c>
       <c r="F53" s="17" t="inlineStr">
@@ -4091,20 +4091,24 @@
       </c>
       <c r="I53" s="9" t="inlineStr">
         <is>
-          <t>Electron is cross-platform; installer, tray and start-at-login need work for each. The 0.6.0 build prompt pack specifies the Linux (.tar.gz and .deb) and macOS (universal .app) builds.</t>
+          <t>One source: a universal macOS app (ad-hoc signed, menu bar, ⌘ menus, Login Items) and Linux .deb and .tar.gz for x64 and arm64 (notifications, autostart, tray-less GNOME handled).</t>
         </is>
       </c>
       <c r="J53" s="15" t="inlineStr">
         <is>
-          <t>Later</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K53" s="17" t="inlineStr">
         <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="L53" s="17" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L53" s="17" t="inlineStr">
+        <is>
+          <t>Implemented in 0.9.0</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="15" t="n">
@@ -4740,9 +4744,67 @@
         </is>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" s="15" t="n">
+        <v>61</v>
+      </c>
+      <c r="B65" s="9" t="inlineStr">
+        <is>
+          <t>Requested in 0.9.1</t>
+        </is>
+      </c>
+      <c r="C65" s="18" t="inlineStr">
+        <is>
+          <t>New (not in the add-on)</t>
+        </is>
+      </c>
+      <c r="D65" s="9" t="inlineStr">
+        <is>
+          <t>Import .ics files whose dates other programs write their own way</t>
+        </is>
+      </c>
+      <c r="E65" s="9" t="inlineStr">
+        <is>
+          <t>Done in 0.9.1</t>
+        </is>
+      </c>
+      <c r="F65" s="17" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="G65" s="10">
+        <f>IFERROR(INDEX(Summary!$B$5:$B$11,MATCH(F65,Summary!$A$5:$A$11,0)),"")</f>
+        <v/>
+      </c>
+      <c r="H65" s="10">
+        <f>IFERROR(INDEX(Summary!$C$5:$C$11,MATCH(F65,Summary!$A$5:$A$11,0)),"")</f>
+        <v/>
+      </c>
+      <c r="I65" s="9" t="inlineStr">
+        <is>
+          <t>"Tue Oct 20 2026 10:00:00 GMT-0400", e-mail dates and 2026-10-20 are read and saved the iCalendar way; an unreadable date is left out instead of stopping the import ("Could not extract integer from "Tue "").</t>
+        </is>
+      </c>
+      <c r="J65" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K65" s="17" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L65" s="17" t="inlineStr">
+        <is>
+          <t>Implemented in 0.9.1</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:L64"/>
-  <conditionalFormatting sqref="F5:F64">
+  <autoFilter ref="A4:L65"/>
+  <conditionalFormatting sqref="F5:F65">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Easy"</formula>
     </cfRule>
@@ -4765,22 +4827,22 @@
       <formula>"Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:L64">
+  <conditionalFormatting sqref="A5:L65">
     <cfRule type="expression" priority="8" dxfId="7">
       <formula>$K5="Done"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation sqref="F5:F64" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F5:F65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Easy,Easy–Medium,Medium,Medium–Hard,Hard,Very hard,Not applicable"</formula1>
     </dataValidation>
-    <dataValidation sqref="K5:K64" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K5:K65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not started,Planned,In progress,Done,Won't do"</formula1>
     </dataValidation>
-    <dataValidation sqref="J5:J64" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J5:J65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"1,2,3,4,Later,—"</formula1>
     </dataValidation>
-    <dataValidation sqref="C5:C64" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="C5:C65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"In ReminderFox 2.1.6,New (not in the add-on)"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4794,7 +4856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4805,7 +4867,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>What ReminderFoxAgain 0.8.1 adds alongside ReminderFox's features</t>
+          <t>What ReminderFoxAgain 0.9.1 adds alongside ReminderFox's features</t>
         </is>
       </c>
     </row>
@@ -4982,10 +5044,25 @@
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
+          <t>Platforms</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>Windows, macOS (one app for Apple silicon and Intel) and Linux (.deb and .tar.gz) from one source, each with its own wording, shortcuts and menus (0.9.0).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
           <t>Installer and tests</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C15" s="9" t="inlineStr">
         <is>
           <t>A per-user installer with checksums and rollback, identical builds, and automated tests (unit, UI, installer).</t>
         </is>

</xml_diff>

<commit_message>
README: feature gaps with the original add-on, and what the app adds
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KZ8RpfjgQtZthigNSkA5xL
</commit_message>
<xml_diff>
--- a/docs/feature-gaps.xlsx
+++ b/docs/feature-gaps.xlsx
@@ -4010,7 +4010,7 @@
       </c>
       <c r="D52" s="9" t="inlineStr">
         <is>
-          <t>35 languages</t>
+          <t>34 languages</t>
         </is>
       </c>
       <c r="E52" s="9" t="inlineStr">
@@ -4033,7 +4033,7 @@
       </c>
       <c r="I52" s="9" t="inlineStr">
         <is>
-          <t>The add-on's languages (English plus 33), following the Windows language by default, with a Language setting in Settings → Display; Arabic and Hebrew right to left; date pickers follow too. The translations were written for ReminderFoxAgain and have not yet been checked by native speakers.</t>
+          <t>The add-on's languages (English plus 33), following the system language by default, with a Language setting in Settings → Display; Arabic and Hebrew right to left; date pickers follow too. The translations were written for ReminderFoxAgain and have not yet been checked by native speakers.</t>
         </is>
       </c>
       <c r="J52" s="15" t="inlineStr">

</xml_diff>

<commit_message>
ReminderFoxAgain 0.9.2: a standard Windows installer (NSIS)
- One file, ReminderFoxAgain-Setup-<ver>.exe, built on Linux with makensis: per user, no admin, same install folder,
  updates .bat-era installs in place, swaps folders with rollback, shortcuts and a Settings -> Apps entry
- A real uninstaller in the app's languages; asks before deleting your reminders (No by default; /S keeps them)
- No PowerShell, execution-policy bypass, part joining or Unblock-File
- tools/test-installer.sh (Wine) replaces tools/test-setup.sh; docs, build prompt pack and feature gaps updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KZ8RpfjgQtZthigNSkA5xL
</commit_message>
<xml_diff>
--- a/docs/feature-gaps.xlsx
+++ b/docs/feature-gaps.xlsx
@@ -1275,7 +1275,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>The original ReminderFox add-on (2.1.6) and ReminderFoxAgain 0.9.1 — ReminderFox's features still to bring across, and new features (proposed or added)</t>
+          <t>The original ReminderFox add-on (2.1.6) and ReminderFoxAgain 0.9.2 — ReminderFox's features still to bring across, and new features (proposed or added)</t>
         </is>
       </c>
     </row>
@@ -1309,7 +1309,7 @@
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>Current app (0.9.1)</t>
+          <t>Current app (0.9.2)</t>
         </is>
       </c>
       <c r="F4" s="14" t="inlineStr">
@@ -4867,7 +4867,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>What ReminderFoxAgain 0.9.1 adds alongside ReminderFox's features</t>
+          <t>What ReminderFoxAgain 0.9.2 adds alongside ReminderFox's features</t>
         </is>
       </c>
     </row>
@@ -5064,7 +5064,7 @@
       </c>
       <c r="C15" s="9" t="inlineStr">
         <is>
-          <t>A per-user installer with checksums and rollback, identical builds, and automated tests (unit, UI, installer).</t>
+          <t>A standard per-user Windows installer (NSIS) with a proper uninstaller, Linux packages and a universal macOS app, identical builds, and automated tests (unit, UI, installer).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Roll back to 0.9.1 (revert "ReminderFoxAgain 0.9.2: a standard Windows installer (NSIS)")
This reverts commit a60d11e: Windows goes back to the .bat + PowerShell setup of 0.9.1. The NSIS installer
remains in the history at a60d11e if it's wanted later.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KZ8RpfjgQtZthigNSkA5xL
</commit_message>
<xml_diff>
--- a/docs/feature-gaps.xlsx
+++ b/docs/feature-gaps.xlsx
@@ -1275,7 +1275,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>The original ReminderFox add-on (2.1.6) and ReminderFoxAgain 0.9.2 — ReminderFox's features still to bring across, and new features (proposed or added)</t>
+          <t>The original ReminderFox add-on (2.1.6) and ReminderFoxAgain 0.9.1 — ReminderFox's features still to bring across, and new features (proposed or added)</t>
         </is>
       </c>
     </row>
@@ -1309,7 +1309,7 @@
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>Current app (0.9.2)</t>
+          <t>Current app (0.9.1)</t>
         </is>
       </c>
       <c r="F4" s="14" t="inlineStr">
@@ -4867,7 +4867,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>What ReminderFoxAgain 0.9.2 adds alongside ReminderFox's features</t>
+          <t>What ReminderFoxAgain 0.9.1 adds alongside ReminderFox's features</t>
         </is>
       </c>
     </row>
@@ -5064,7 +5064,7 @@
       </c>
       <c r="C15" s="9" t="inlineStr">
         <is>
-          <t>A standard per-user Windows installer (NSIS) with a proper uninstaller, Linux packages and a universal macOS app, identical builds, and automated tests (unit, UI, installer).</t>
+          <t>A per-user installer with checksums and rollback, identical builds, and automated tests (unit, UI, installer).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ReminderFoxAgain 0.9.2: fits the smallest window
- Version 0.9.2 in package.json, package-lock.json, the README, the docs,
  the build prompt pack (Android/iOS build 902) and feature-gaps.xlsx.
- CHANGELOG and README "What's new": the 820 px layout fix.
- User's Guide: what a narrow window looks like. Technical System
  Design: a "Narrow windows (0.9.2)" section. Developer's Guide and the
  build prompt: the layout checks at 820 px and the new e2e counts
  (658 checks in 37 runs).
- docs/*.md and docs/word/*.docx exported again from the Claude Docs.
- README pictures: the status bar shows 0.9.2 (nothing else changed;
  the app looks the same at 1180 px).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JJP6L9dU2itRAGFeJexq3u
</commit_message>
<xml_diff>
--- a/docs/feature-gaps.xlsx
+++ b/docs/feature-gaps.xlsx
@@ -1275,7 +1275,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>The original ReminderFox add-on (2.1.6) and ReminderFoxAgain 0.9.1 — ReminderFox's features still to bring across, and new features (proposed or added)</t>
+          <t>The original ReminderFox add-on (2.1.6) and ReminderFoxAgain 0.9.2 — ReminderFox's features still to bring across, and new features (proposed or added)</t>
         </is>
       </c>
     </row>
@@ -1309,7 +1309,7 @@
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>Current app (0.9.1)</t>
+          <t>Current app (0.9.2)</t>
         </is>
       </c>
       <c r="F4" s="14" t="inlineStr">
@@ -4867,7 +4867,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>What ReminderFoxAgain 0.9.1 adds alongside ReminderFox's features</t>
+          <t>What ReminderFoxAgain 0.9.2 adds alongside ReminderFox's features</t>
         </is>
       </c>
     </row>

</xml_diff>